<commit_message>
added some more wcag mappings and recommendations
</commit_message>
<xml_diff>
--- a/Analysis_Output/Final_excel_generated.xlsx
+++ b/Analysis_Output/Final_excel_generated.xlsx
@@ -137,8 +137,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="FinalSummaryTable" displayName="FinalSummaryTable" ref="A1:D6" headerRowCount="1">
-  <autoFilter ref="A1:D6"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="FinalSummaryTable" displayName="FinalSummaryTable" ref="A1:D17" headerRowCount="1">
+  <autoFilter ref="A1:D17"/>
   <tableColumns count="4">
     <tableColumn id="1" name="filename"/>
     <tableColumn id="2" name="categorization"/>
@@ -438,11 +438,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:D17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="17" customWidth="1" min="2" max="2"/>
     <col width="34" customWidth="1" min="3" max="3"/>
     <col width="15" customWidth="1" min="4" max="4"/>
   </cols>
@@ -472,17 +472,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>CCP1000.pdf</t>
+          <t>CCJ0700.pdf</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>PDFforms</t>
+          <t>PDF with images</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Final_report_excels\CCP1000.xlsx</t>
+          <t>Final_report_excels\CCJ0700.xlsx</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -494,7 +494,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>CCP1003.pdf</t>
+          <t>CCG0134.pdf</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -504,7 +504,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Final_report_excels\CCP1003.xlsx</t>
+          <t>Final_report_excels\CCG0134.xlsx</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -516,7 +516,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>CCP1004.pdf</t>
+          <t>CCG0135.pdf</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -526,7 +526,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Final_report_excels\CCP1004.xlsx</t>
+          <t>Final_report_excels\CCG0135.xlsx</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -538,7 +538,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>CCP1005.pdf</t>
+          <t>CCG0136.pdf</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -548,7 +548,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Final_report_excels\CCP1005.xlsx</t>
+          <t>Final_report_excels\CCG0136.xlsx</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -560,7 +560,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>CCP1007.pdf</t>
+          <t>CCG0137.pdf</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -570,12 +570,254 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Final_report_excels\CCP1007.xlsx</t>
+          <t>Final_report_excels\CCG0137.xlsx</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
           <t>Large</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>CCG0813.pdf</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>PDFforms</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Final_report_excels\CCG0813.xlsx</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>CCG0650.pdf</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>PDFforms</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Final_report_excels\CCG0650.xlsx</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>CCG0125.pdf</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>PDFforms</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Final_report_excels\CCG0125.xlsx</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Small</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>CCJ0031.pdf</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>PDFforms</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Final_report_excels\CCJ0031.xlsx</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Small</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>CCG0613.pdf</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>PDFforms</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Final_report_excels\CCG0613.xlsx</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Small</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>CCG0646.pdf</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>PDFforms</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Final_report_excels\CCG0646.xlsx</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Small</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>CCG0815.pdf</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>PDFforms</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Final_report_excels\CCG0815.xlsx</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Small</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>GCR2403.pdf</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Pdf</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Final_report_excels\GCR2403.xlsx</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Small</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>IRP1101.pdf</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Pdf</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Final_report_excels\IRP1101.xlsx</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Small</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>MNO705.pdf</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Pdf</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Final_report_excels\MNO705.xlsx</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Small</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>MSA902.pdf</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Pdf</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Final_report_excels\MSA902.xlsx</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Small</t>
         </is>
       </c>
     </row>

</xml_diff>